<commit_message>
Generert PDF av skjematikken
</commit_message>
<xml_diff>
--- a/common/TPS26400 - Design Calculator.xlsx
+++ b/common/TPS26400 - Design Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vikin\Documents\KybStudie\Vortex\vortex-newtype-drone-PCBs\common\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51A3967A-3543-48E7-AB81-0BE819E7C9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57FF66F-F31D-4BDF-A871-B4543EA9DAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10776" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculation Sheet" sheetId="1" r:id="rId1"/>
@@ -1884,23 +1884,23 @@
     <xf numFmtId="0" fontId="28" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2044,13 +2044,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>12.588888888888887</c:v>
+                  <c:v>13.123255813953486</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.618888888888888</c:v>
+                  <c:v>14.196976744186045</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.428333333333335</c:v>
+                  <c:v>20.349</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4196,7 +4196,7 @@
         <v>71</v>
       </c>
       <c r="D6" s="52">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="53" t="s">
         <v>6</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="D16" s="59">
         <f>D15*((UVLOref*OVset/(UVset*OVPref))-1)</f>
-        <v>16.15384615384615</v>
+        <v>12.857142857142851</v>
       </c>
       <c r="E16" s="60" t="s">
         <v>68</v>
@@ -4343,14 +4343,14 @@
       <c r="F16" s="14"/>
       <c r="J16" s="3">
         <f>D24</f>
-        <v>12.588888888888887</v>
+        <v>13.123255813953486</v>
       </c>
       <c r="K16" s="35" t="s">
         <v>55</v>
       </c>
       <c r="M16" s="1">
         <f t="shared" ref="M16:M17" si="0">IF(D16&lt;10, D16*100, IF(AND(D16&gt;=10, D16&lt;100),D16*10,IF(AND(D16&gt;=100, D16&lt;1000), D16, IF(D16&gt;=1000, D16/10))))</f>
-        <v>161.53846153846149</v>
+        <v>128.5714285714285</v>
       </c>
     </row>
     <row r="17" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="D17" s="59">
         <f>D15*(OVset/OVPref)*(1-(UVLOref/UVset))</f>
-        <v>458.04783451842275</v>
+        <v>461.3445378151261</v>
       </c>
       <c r="E17" s="60" t="s">
         <v>68</v>
@@ -4370,14 +4370,14 @@
       <c r="F17" s="14"/>
       <c r="J17" s="3">
         <f>D22</f>
-        <v>13.618888888888888</v>
+        <v>14.196976744186045</v>
       </c>
       <c r="K17" s="35" t="s">
         <v>56</v>
       </c>
       <c r="M17" s="1">
         <f t="shared" si="0"/>
-        <v>458.04783451842275</v>
+        <v>461.3445378151261</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4390,7 +4390,7 @@
       <c r="F18" s="11"/>
       <c r="J18" s="3">
         <f>D23</f>
-        <v>20.428333333333335</v>
+        <v>20.349</v>
       </c>
       <c r="K18" s="35" t="s">
         <v>167</v>
@@ -4430,7 +4430,7 @@
         <v>136</v>
       </c>
       <c r="D20" s="120">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E20" s="60" t="s">
         <v>68</v>
@@ -4441,11 +4441,11 @@
       </c>
       <c r="G20" s="15">
         <f>M20*D16/M16</f>
-        <v>16.2</v>
+        <v>13.000000000000002</v>
       </c>
       <c r="M20" s="47">
         <f>INDEX('Res EIA Tables'!E$5:E$196,2+MATCH(M16,'Res EIA Tables'!E$5:E$196))</f>
-        <v>162</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="G21" s="48">
         <f>M21*D17/M17</f>
-        <v>464</v>
+        <v>463.99999999999994</v>
       </c>
       <c r="M21" s="47">
         <f>INDEX('Res EIA Tables'!E$5:E$196,2+MATCH(M17,'Res EIA Tables'!E$5:E$196))</f>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="D22" s="63">
         <f>UVLOref*((ROVP+RUVLO+RIN)/(ROVP+RUVLO))</f>
-        <v>13.618888888888888</v>
+        <v>14.196976744186045</v>
       </c>
       <c r="E22" s="64" t="s">
         <v>6</v>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="D23" s="63">
         <f>OVPref*((ROVP+RUVLO+RIN)/ROVP)</f>
-        <v>20.428333333333335</v>
+        <v>20.349</v>
       </c>
       <c r="E23" s="64" t="s">
         <v>6</v>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="D24" s="63">
         <f>(UVLOref-UVLOhys)*((ROVP+RUVLO+RIN)/(ROVP+RUVLO))</f>
-        <v>12.588888888888887</v>
+        <v>13.123255813953486</v>
       </c>
       <c r="E24" s="64" t="s">
         <v>6</v>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="D25" s="65">
         <f>Vinmax*1000/(ROVP+RUVLO+RIN)</f>
-        <v>46.601941747572816</v>
+        <v>46.783625730994153</v>
       </c>
       <c r="E25" s="60" t="s">
         <v>7</v>
@@ -6644,14 +6644,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="141" t="s">
+      <c r="A1" s="143" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="141"/>
-      <c r="C1" s="141"/>
-      <c r="D1" s="141"/>
-      <c r="E1" s="141"/>
-      <c r="F1" s="141"/>
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
@@ -6697,16 +6697,16 @@
       <c r="A5" s="142">
         <v>100</v>
       </c>
-      <c r="B5" s="143">
+      <c r="B5" s="140">
         <v>100</v>
       </c>
-      <c r="C5" s="138">
+      <c r="C5" s="141">
         <v>100</v>
       </c>
       <c r="D5" s="139">
         <v>100</v>
       </c>
-      <c r="E5" s="140">
+      <c r="E5" s="138">
         <v>100</v>
       </c>
       <c r="F5" s="8">
@@ -6715,20 +6715,20 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="142"/>
-      <c r="B6" s="143"/>
-      <c r="C6" s="138"/>
+      <c r="B6" s="140"/>
+      <c r="C6" s="141"/>
       <c r="D6" s="139"/>
-      <c r="E6" s="140"/>
+      <c r="E6" s="138"/>
       <c r="F6" s="8">
         <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="142"/>
-      <c r="B7" s="143"/>
-      <c r="C7" s="138"/>
+      <c r="B7" s="140"/>
+      <c r="C7" s="141"/>
       <c r="D7" s="139"/>
-      <c r="E7" s="140">
+      <c r="E7" s="138">
         <v>102</v>
       </c>
       <c r="F7" s="8">
@@ -6737,22 +6737,22 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="142"/>
-      <c r="B8" s="143"/>
-      <c r="C8" s="138"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="141"/>
       <c r="D8" s="139"/>
-      <c r="E8" s="140"/>
+      <c r="E8" s="138"/>
       <c r="F8" s="8">
         <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="142"/>
-      <c r="B9" s="143"/>
-      <c r="C9" s="138"/>
+      <c r="B9" s="140"/>
+      <c r="C9" s="141"/>
       <c r="D9" s="139">
         <v>105</v>
       </c>
-      <c r="E9" s="140">
+      <c r="E9" s="138">
         <v>105</v>
       </c>
       <c r="F9" s="8">
@@ -6761,10 +6761,10 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="142"/>
-      <c r="B10" s="143"/>
-      <c r="C10" s="138"/>
+      <c r="B10" s="140"/>
+      <c r="C10" s="141"/>
       <c r="D10" s="139"/>
-      <c r="E10" s="140"/>
+      <c r="E10" s="138"/>
       <c r="F10" s="8">
         <v>106</v>
       </c>
@@ -6772,10 +6772,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="142"/>
-      <c r="B11" s="143"/>
-      <c r="C11" s="138"/>
+      <c r="B11" s="140"/>
+      <c r="C11" s="141"/>
       <c r="D11" s="139"/>
-      <c r="E11" s="140">
+      <c r="E11" s="138">
         <v>107</v>
       </c>
       <c r="F11" s="8">
@@ -6784,24 +6784,24 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="142"/>
-      <c r="B12" s="143"/>
-      <c r="C12" s="138"/>
+      <c r="B12" s="140"/>
+      <c r="C12" s="141"/>
       <c r="D12" s="139"/>
-      <c r="E12" s="140"/>
+      <c r="E12" s="138"/>
       <c r="F12" s="8">
         <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="142"/>
-      <c r="B13" s="143"/>
-      <c r="C13" s="138">
+      <c r="B13" s="140"/>
+      <c r="C13" s="141">
         <v>110</v>
       </c>
       <c r="D13" s="139">
         <v>110</v>
       </c>
-      <c r="E13" s="140">
+      <c r="E13" s="138">
         <v>110</v>
       </c>
       <c r="F13" s="8">
@@ -6810,20 +6810,20 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="142"/>
-      <c r="B14" s="143"/>
-      <c r="C14" s="138"/>
+      <c r="B14" s="140"/>
+      <c r="C14" s="141"/>
       <c r="D14" s="139"/>
-      <c r="E14" s="140"/>
+      <c r="E14" s="138"/>
       <c r="F14" s="8">
         <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="142"/>
-      <c r="B15" s="143"/>
-      <c r="C15" s="138"/>
+      <c r="B15" s="140"/>
+      <c r="C15" s="141"/>
       <c r="D15" s="139"/>
-      <c r="E15" s="140">
+      <c r="E15" s="138">
         <v>113</v>
       </c>
       <c r="F15" s="8">
@@ -6832,22 +6832,22 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="142"/>
-      <c r="B16" s="143"/>
-      <c r="C16" s="138"/>
+      <c r="B16" s="140"/>
+      <c r="C16" s="141"/>
       <c r="D16" s="139"/>
-      <c r="E16" s="140"/>
+      <c r="E16" s="138"/>
       <c r="F16" s="8">
         <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="142"/>
-      <c r="B17" s="143"/>
-      <c r="C17" s="138"/>
+      <c r="B17" s="140"/>
+      <c r="C17" s="141"/>
       <c r="D17" s="139">
         <v>115</v>
       </c>
-      <c r="E17" s="140">
+      <c r="E17" s="138">
         <v>115</v>
       </c>
       <c r="F17" s="8">
@@ -6856,20 +6856,20 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="142"/>
-      <c r="B18" s="143"/>
-      <c r="C18" s="138"/>
+      <c r="B18" s="140"/>
+      <c r="C18" s="141"/>
       <c r="D18" s="139"/>
-      <c r="E18" s="140"/>
+      <c r="E18" s="138"/>
       <c r="F18" s="8">
         <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="142"/>
-      <c r="B19" s="143"/>
-      <c r="C19" s="138"/>
+      <c r="B19" s="140"/>
+      <c r="C19" s="141"/>
       <c r="D19" s="139"/>
-      <c r="E19" s="140">
+      <c r="E19" s="138">
         <v>118</v>
       </c>
       <c r="F19" s="8">
@@ -6878,26 +6878,26 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="142"/>
-      <c r="B20" s="143"/>
-      <c r="C20" s="138"/>
+      <c r="B20" s="140"/>
+      <c r="C20" s="141"/>
       <c r="D20" s="139"/>
-      <c r="E20" s="140"/>
+      <c r="E20" s="138"/>
       <c r="F20" s="8">
         <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="142"/>
-      <c r="B21" s="143">
+      <c r="B21" s="140">
         <v>120</v>
       </c>
-      <c r="C21" s="138">
+      <c r="C21" s="141">
         <v>120</v>
       </c>
       <c r="D21" s="139">
         <v>121</v>
       </c>
-      <c r="E21" s="140">
+      <c r="E21" s="138">
         <v>121</v>
       </c>
       <c r="F21" s="8">
@@ -6906,20 +6906,20 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="142"/>
-      <c r="B22" s="143"/>
-      <c r="C22" s="138"/>
+      <c r="B22" s="140"/>
+      <c r="C22" s="141"/>
       <c r="D22" s="139"/>
-      <c r="E22" s="140"/>
+      <c r="E22" s="138"/>
       <c r="F22" s="8">
         <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="142"/>
-      <c r="B23" s="143"/>
-      <c r="C23" s="138"/>
+      <c r="B23" s="140"/>
+      <c r="C23" s="141"/>
       <c r="D23" s="139"/>
-      <c r="E23" s="140">
+      <c r="E23" s="138">
         <v>124</v>
       </c>
       <c r="F23" s="8">
@@ -6928,22 +6928,22 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="142"/>
-      <c r="B24" s="143"/>
-      <c r="C24" s="138"/>
+      <c r="B24" s="140"/>
+      <c r="C24" s="141"/>
       <c r="D24" s="139"/>
-      <c r="E24" s="140"/>
+      <c r="E24" s="138"/>
       <c r="F24" s="8">
         <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="142"/>
-      <c r="B25" s="143"/>
-      <c r="C25" s="138"/>
+      <c r="B25" s="140"/>
+      <c r="C25" s="141"/>
       <c r="D25" s="139">
         <v>127</v>
       </c>
-      <c r="E25" s="140">
+      <c r="E25" s="138">
         <v>127</v>
       </c>
       <c r="F25" s="8">
@@ -6952,20 +6952,20 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="142"/>
-      <c r="B26" s="143"/>
-      <c r="C26" s="138"/>
+      <c r="B26" s="140"/>
+      <c r="C26" s="141"/>
       <c r="D26" s="139"/>
-      <c r="E26" s="140"/>
+      <c r="E26" s="138"/>
       <c r="F26" s="8">
         <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="142"/>
-      <c r="B27" s="143"/>
-      <c r="C27" s="138"/>
+      <c r="B27" s="140"/>
+      <c r="C27" s="141"/>
       <c r="D27" s="139"/>
-      <c r="E27" s="140">
+      <c r="E27" s="138">
         <v>130</v>
       </c>
       <c r="F27" s="8">
@@ -6974,24 +6974,24 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="142"/>
-      <c r="B28" s="143"/>
-      <c r="C28" s="138"/>
+      <c r="B28" s="140"/>
+      <c r="C28" s="141"/>
       <c r="D28" s="139"/>
-      <c r="E28" s="140"/>
+      <c r="E28" s="138"/>
       <c r="F28" s="8">
         <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="142"/>
-      <c r="B29" s="143"/>
-      <c r="C29" s="138">
+      <c r="B29" s="140"/>
+      <c r="C29" s="141">
         <v>130</v>
       </c>
       <c r="D29" s="139">
         <v>133</v>
       </c>
-      <c r="E29" s="140">
+      <c r="E29" s="138">
         <v>133</v>
       </c>
       <c r="F29" s="8">
@@ -7000,20 +7000,20 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="142"/>
-      <c r="B30" s="143"/>
-      <c r="C30" s="138"/>
+      <c r="B30" s="140"/>
+      <c r="C30" s="141"/>
       <c r="D30" s="139"/>
-      <c r="E30" s="140"/>
+      <c r="E30" s="138"/>
       <c r="F30" s="8">
         <v>135</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="142"/>
-      <c r="B31" s="143"/>
-      <c r="C31" s="138"/>
+      <c r="B31" s="140"/>
+      <c r="C31" s="141"/>
       <c r="D31" s="139"/>
-      <c r="E31" s="140">
+      <c r="E31" s="138">
         <v>137</v>
       </c>
       <c r="F31" s="8">
@@ -7022,22 +7022,22 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="142"/>
-      <c r="B32" s="143"/>
-      <c r="C32" s="138"/>
+      <c r="B32" s="140"/>
+      <c r="C32" s="141"/>
       <c r="D32" s="139"/>
-      <c r="E32" s="140"/>
+      <c r="E32" s="138"/>
       <c r="F32" s="8">
         <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="142"/>
-      <c r="B33" s="143"/>
-      <c r="C33" s="138"/>
+      <c r="B33" s="140"/>
+      <c r="C33" s="141"/>
       <c r="D33" s="139">
         <v>140</v>
       </c>
-      <c r="E33" s="140">
+      <c r="E33" s="138">
         <v>140</v>
       </c>
       <c r="F33" s="8">
@@ -7046,20 +7046,20 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="142"/>
-      <c r="B34" s="143"/>
-      <c r="C34" s="138"/>
+      <c r="B34" s="140"/>
+      <c r="C34" s="141"/>
       <c r="D34" s="139"/>
-      <c r="E34" s="140"/>
+      <c r="E34" s="138"/>
       <c r="F34" s="8">
         <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="142"/>
-      <c r="B35" s="143"/>
-      <c r="C35" s="138"/>
+      <c r="B35" s="140"/>
+      <c r="C35" s="141"/>
       <c r="D35" s="139"/>
-      <c r="E35" s="140">
+      <c r="E35" s="138">
         <v>143</v>
       </c>
       <c r="F35" s="8">
@@ -7068,10 +7068,10 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="142"/>
-      <c r="B36" s="143"/>
-      <c r="C36" s="138"/>
+      <c r="B36" s="140"/>
+      <c r="C36" s="141"/>
       <c r="D36" s="139"/>
-      <c r="E36" s="140"/>
+      <c r="E36" s="138"/>
       <c r="F36" s="8">
         <v>145</v>
       </c>
@@ -7080,16 +7080,16 @@
       <c r="A37" s="142">
         <v>150</v>
       </c>
-      <c r="B37" s="143">
+      <c r="B37" s="140">
         <v>150</v>
       </c>
-      <c r="C37" s="138">
+      <c r="C37" s="141">
         <v>150</v>
       </c>
       <c r="D37" s="139">
         <v>147</v>
       </c>
-      <c r="E37" s="140">
+      <c r="E37" s="138">
         <v>147</v>
       </c>
       <c r="F37" s="8">
@@ -7098,20 +7098,20 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="142"/>
-      <c r="B38" s="143"/>
-      <c r="C38" s="138"/>
+      <c r="B38" s="140"/>
+      <c r="C38" s="141"/>
       <c r="D38" s="139"/>
-      <c r="E38" s="140"/>
+      <c r="E38" s="138"/>
       <c r="F38" s="8">
         <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="142"/>
-      <c r="B39" s="143"/>
-      <c r="C39" s="138"/>
+      <c r="B39" s="140"/>
+      <c r="C39" s="141"/>
       <c r="D39" s="139"/>
-      <c r="E39" s="140">
+      <c r="E39" s="138">
         <v>150</v>
       </c>
       <c r="F39" s="8">
@@ -7120,22 +7120,22 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="142"/>
-      <c r="B40" s="143"/>
-      <c r="C40" s="138"/>
+      <c r="B40" s="140"/>
+      <c r="C40" s="141"/>
       <c r="D40" s="139"/>
-      <c r="E40" s="140"/>
+      <c r="E40" s="138"/>
       <c r="F40" s="8">
         <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="142"/>
-      <c r="B41" s="143"/>
-      <c r="C41" s="138"/>
+      <c r="B41" s="140"/>
+      <c r="C41" s="141"/>
       <c r="D41" s="139">
         <v>154</v>
       </c>
-      <c r="E41" s="140">
+      <c r="E41" s="138">
         <v>154</v>
       </c>
       <c r="F41" s="8">
@@ -7144,20 +7144,20 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="142"/>
-      <c r="B42" s="143"/>
-      <c r="C42" s="138"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="141"/>
       <c r="D42" s="139"/>
-      <c r="E42" s="140"/>
+      <c r="E42" s="138"/>
       <c r="F42" s="8">
         <v>156</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="142"/>
-      <c r="B43" s="143"/>
-      <c r="C43" s="138"/>
+      <c r="B43" s="140"/>
+      <c r="C43" s="141"/>
       <c r="D43" s="139"/>
-      <c r="E43" s="140">
+      <c r="E43" s="138">
         <v>158</v>
       </c>
       <c r="F43" s="8">
@@ -7166,24 +7166,24 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="142"/>
-      <c r="B44" s="143"/>
-      <c r="C44" s="138"/>
+      <c r="B44" s="140"/>
+      <c r="C44" s="141"/>
       <c r="D44" s="139"/>
-      <c r="E44" s="140"/>
+      <c r="E44" s="138"/>
       <c r="F44" s="8">
         <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="142"/>
-      <c r="B45" s="143"/>
-      <c r="C45" s="138">
+      <c r="B45" s="140"/>
+      <c r="C45" s="141">
         <v>160</v>
       </c>
       <c r="D45" s="139">
         <v>162</v>
       </c>
-      <c r="E45" s="140">
+      <c r="E45" s="138">
         <v>162</v>
       </c>
       <c r="F45" s="8">
@@ -7192,20 +7192,20 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="142"/>
-      <c r="B46" s="143"/>
-      <c r="C46" s="138"/>
+      <c r="B46" s="140"/>
+      <c r="C46" s="141"/>
       <c r="D46" s="139"/>
-      <c r="E46" s="140"/>
+      <c r="E46" s="138"/>
       <c r="F46" s="8">
         <v>164</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="142"/>
-      <c r="B47" s="143"/>
-      <c r="C47" s="138"/>
+      <c r="B47" s="140"/>
+      <c r="C47" s="141"/>
       <c r="D47" s="139"/>
-      <c r="E47" s="140">
+      <c r="E47" s="138">
         <v>165</v>
       </c>
       <c r="F47" s="8">
@@ -7214,22 +7214,22 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="142"/>
-      <c r="B48" s="143"/>
-      <c r="C48" s="138"/>
+      <c r="B48" s="140"/>
+      <c r="C48" s="141"/>
       <c r="D48" s="139"/>
-      <c r="E48" s="140"/>
+      <c r="E48" s="138"/>
       <c r="F48" s="8">
         <v>167</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="142"/>
-      <c r="B49" s="143"/>
-      <c r="C49" s="138"/>
+      <c r="B49" s="140"/>
+      <c r="C49" s="141"/>
       <c r="D49" s="139">
         <v>169</v>
       </c>
-      <c r="E49" s="140">
+      <c r="E49" s="138">
         <v>169</v>
       </c>
       <c r="F49" s="8">
@@ -7238,20 +7238,20 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="142"/>
-      <c r="B50" s="143"/>
-      <c r="C50" s="138"/>
+      <c r="B50" s="140"/>
+      <c r="C50" s="141"/>
       <c r="D50" s="139"/>
-      <c r="E50" s="140"/>
+      <c r="E50" s="138"/>
       <c r="F50" s="8">
         <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="142"/>
-      <c r="B51" s="143"/>
-      <c r="C51" s="138"/>
+      <c r="B51" s="140"/>
+      <c r="C51" s="141"/>
       <c r="D51" s="139"/>
-      <c r="E51" s="140">
+      <c r="E51" s="138">
         <v>174</v>
       </c>
       <c r="F51" s="8">
@@ -7260,26 +7260,26 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="142"/>
-      <c r="B52" s="143"/>
-      <c r="C52" s="138"/>
+      <c r="B52" s="140"/>
+      <c r="C52" s="141"/>
       <c r="D52" s="139"/>
-      <c r="E52" s="140"/>
+      <c r="E52" s="138"/>
       <c r="F52" s="8">
         <v>176</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="142"/>
-      <c r="B53" s="143">
+      <c r="B53" s="140">
         <v>180</v>
       </c>
-      <c r="C53" s="138">
+      <c r="C53" s="141">
         <v>180</v>
       </c>
       <c r="D53" s="139">
         <v>178</v>
       </c>
-      <c r="E53" s="140">
+      <c r="E53" s="138">
         <v>178</v>
       </c>
       <c r="F53" s="8">
@@ -7288,20 +7288,20 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="142"/>
-      <c r="B54" s="143"/>
-      <c r="C54" s="138"/>
+      <c r="B54" s="140"/>
+      <c r="C54" s="141"/>
       <c r="D54" s="139"/>
-      <c r="E54" s="140"/>
+      <c r="E54" s="138"/>
       <c r="F54" s="8">
         <v>180</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="142"/>
-      <c r="B55" s="143"/>
-      <c r="C55" s="138"/>
+      <c r="B55" s="140"/>
+      <c r="C55" s="141"/>
       <c r="D55" s="139"/>
-      <c r="E55" s="140">
+      <c r="E55" s="138">
         <v>182</v>
       </c>
       <c r="F55" s="8">
@@ -7310,22 +7310,22 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="142"/>
-      <c r="B56" s="143"/>
-      <c r="C56" s="138"/>
+      <c r="B56" s="140"/>
+      <c r="C56" s="141"/>
       <c r="D56" s="139"/>
-      <c r="E56" s="140"/>
+      <c r="E56" s="138"/>
       <c r="F56" s="8">
         <v>184</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="142"/>
-      <c r="B57" s="143"/>
-      <c r="C57" s="138"/>
+      <c r="B57" s="140"/>
+      <c r="C57" s="141"/>
       <c r="D57" s="139">
         <v>187</v>
       </c>
-      <c r="E57" s="140">
+      <c r="E57" s="138">
         <v>187</v>
       </c>
       <c r="F57" s="8">
@@ -7334,20 +7334,20 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="142"/>
-      <c r="B58" s="143"/>
-      <c r="C58" s="138"/>
+      <c r="B58" s="140"/>
+      <c r="C58" s="141"/>
       <c r="D58" s="139"/>
-      <c r="E58" s="140"/>
+      <c r="E58" s="138"/>
       <c r="F58" s="8">
         <v>189</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="142"/>
-      <c r="B59" s="143"/>
-      <c r="C59" s="138"/>
+      <c r="B59" s="140"/>
+      <c r="C59" s="141"/>
       <c r="D59" s="139"/>
-      <c r="E59" s="140">
+      <c r="E59" s="138">
         <v>191</v>
       </c>
       <c r="F59" s="8">
@@ -7356,24 +7356,24 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="142"/>
-      <c r="B60" s="143"/>
-      <c r="C60" s="138"/>
+      <c r="B60" s="140"/>
+      <c r="C60" s="141"/>
       <c r="D60" s="139"/>
-      <c r="E60" s="140"/>
+      <c r="E60" s="138"/>
       <c r="F60" s="8">
         <v>193</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="142"/>
-      <c r="B61" s="143"/>
-      <c r="C61" s="138">
+      <c r="B61" s="140"/>
+      <c r="C61" s="141">
         <v>200</v>
       </c>
       <c r="D61" s="139">
         <v>196</v>
       </c>
-      <c r="E61" s="140">
+      <c r="E61" s="138">
         <v>196</v>
       </c>
       <c r="F61" s="8">
@@ -7382,20 +7382,20 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="142"/>
-      <c r="B62" s="143"/>
-      <c r="C62" s="138"/>
+      <c r="B62" s="140"/>
+      <c r="C62" s="141"/>
       <c r="D62" s="139"/>
-      <c r="E62" s="140"/>
+      <c r="E62" s="138"/>
       <c r="F62" s="8">
         <v>198</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="142"/>
-      <c r="B63" s="143"/>
-      <c r="C63" s="138"/>
+      <c r="B63" s="140"/>
+      <c r="C63" s="141"/>
       <c r="D63" s="139"/>
-      <c r="E63" s="140">
+      <c r="E63" s="138">
         <v>200</v>
       </c>
       <c r="F63" s="8">
@@ -7404,22 +7404,22 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="142"/>
-      <c r="B64" s="143"/>
-      <c r="C64" s="138"/>
+      <c r="B64" s="140"/>
+      <c r="C64" s="141"/>
       <c r="D64" s="139"/>
-      <c r="E64" s="140"/>
+      <c r="E64" s="138"/>
       <c r="F64" s="8">
         <v>203</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="142"/>
-      <c r="B65" s="143"/>
-      <c r="C65" s="138"/>
+      <c r="B65" s="140"/>
+      <c r="C65" s="141"/>
       <c r="D65" s="139">
         <v>205</v>
       </c>
-      <c r="E65" s="140">
+      <c r="E65" s="138">
         <v>205</v>
       </c>
       <c r="F65" s="8">
@@ -7428,20 +7428,20 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="142"/>
-      <c r="B66" s="143"/>
-      <c r="C66" s="138"/>
+      <c r="B66" s="140"/>
+      <c r="C66" s="141"/>
       <c r="D66" s="139"/>
-      <c r="E66" s="140"/>
+      <c r="E66" s="138"/>
       <c r="F66" s="8">
         <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="142"/>
-      <c r="B67" s="143"/>
-      <c r="C67" s="138"/>
+      <c r="B67" s="140"/>
+      <c r="C67" s="141"/>
       <c r="D67" s="139"/>
-      <c r="E67" s="140">
+      <c r="E67" s="138">
         <v>210</v>
       </c>
       <c r="F67" s="8">
@@ -7450,10 +7450,10 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="142"/>
-      <c r="B68" s="143"/>
-      <c r="C68" s="138"/>
+      <c r="B68" s="140"/>
+      <c r="C68" s="141"/>
       <c r="D68" s="139"/>
-      <c r="E68" s="140"/>
+      <c r="E68" s="138"/>
       <c r="F68" s="8">
         <v>213</v>
       </c>
@@ -7462,16 +7462,16 @@
       <c r="A69" s="142">
         <v>220</v>
       </c>
-      <c r="B69" s="143">
+      <c r="B69" s="140">
         <v>220</v>
       </c>
-      <c r="C69" s="138">
+      <c r="C69" s="141">
         <v>220</v>
       </c>
       <c r="D69" s="139">
         <v>215</v>
       </c>
-      <c r="E69" s="140">
+      <c r="E69" s="138">
         <v>215</v>
       </c>
       <c r="F69" s="8">
@@ -7480,20 +7480,20 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="142"/>
-      <c r="B70" s="143"/>
-      <c r="C70" s="138"/>
+      <c r="B70" s="140"/>
+      <c r="C70" s="141"/>
       <c r="D70" s="139"/>
-      <c r="E70" s="140"/>
+      <c r="E70" s="138"/>
       <c r="F70" s="8">
         <v>218</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="142"/>
-      <c r="B71" s="143"/>
-      <c r="C71" s="138"/>
+      <c r="B71" s="140"/>
+      <c r="C71" s="141"/>
       <c r="D71" s="139"/>
-      <c r="E71" s="140">
+      <c r="E71" s="138">
         <v>221</v>
       </c>
       <c r="F71" s="8">
@@ -7502,22 +7502,22 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="142"/>
-      <c r="B72" s="143"/>
-      <c r="C72" s="138"/>
+      <c r="B72" s="140"/>
+      <c r="C72" s="141"/>
       <c r="D72" s="139"/>
-      <c r="E72" s="140"/>
+      <c r="E72" s="138"/>
       <c r="F72" s="8">
         <v>223</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="142"/>
-      <c r="B73" s="143"/>
-      <c r="C73" s="138"/>
+      <c r="B73" s="140"/>
+      <c r="C73" s="141"/>
       <c r="D73" s="139">
         <v>226</v>
       </c>
-      <c r="E73" s="140">
+      <c r="E73" s="138">
         <v>226</v>
       </c>
       <c r="F73" s="8">
@@ -7526,20 +7526,20 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="142"/>
-      <c r="B74" s="143"/>
-      <c r="C74" s="138"/>
+      <c r="B74" s="140"/>
+      <c r="C74" s="141"/>
       <c r="D74" s="139"/>
-      <c r="E74" s="140"/>
+      <c r="E74" s="138"/>
       <c r="F74" s="8">
         <v>229</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="142"/>
-      <c r="B75" s="143"/>
-      <c r="C75" s="138"/>
+      <c r="B75" s="140"/>
+      <c r="C75" s="141"/>
       <c r="D75" s="139"/>
-      <c r="E75" s="140">
+      <c r="E75" s="138">
         <v>232</v>
       </c>
       <c r="F75" s="8">
@@ -7548,24 +7548,24 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="142"/>
-      <c r="B76" s="143"/>
-      <c r="C76" s="138"/>
+      <c r="B76" s="140"/>
+      <c r="C76" s="141"/>
       <c r="D76" s="139"/>
-      <c r="E76" s="140"/>
+      <c r="E76" s="138"/>
       <c r="F76" s="8">
         <v>234</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="142"/>
-      <c r="B77" s="143"/>
-      <c r="C77" s="138">
+      <c r="B77" s="140"/>
+      <c r="C77" s="141">
         <v>240</v>
       </c>
       <c r="D77" s="139">
         <v>237</v>
       </c>
-      <c r="E77" s="140">
+      <c r="E77" s="138">
         <v>237</v>
       </c>
       <c r="F77" s="8">
@@ -7574,20 +7574,20 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="142"/>
-      <c r="B78" s="143"/>
-      <c r="C78" s="138"/>
+      <c r="B78" s="140"/>
+      <c r="C78" s="141"/>
       <c r="D78" s="139"/>
-      <c r="E78" s="140"/>
+      <c r="E78" s="138"/>
       <c r="F78" s="8">
         <v>240</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="142"/>
-      <c r="B79" s="143"/>
-      <c r="C79" s="138"/>
+      <c r="B79" s="140"/>
+      <c r="C79" s="141"/>
       <c r="D79" s="139"/>
-      <c r="E79" s="140">
+      <c r="E79" s="138">
         <v>243</v>
       </c>
       <c r="F79" s="8">
@@ -7596,22 +7596,22 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="142"/>
-      <c r="B80" s="143"/>
-      <c r="C80" s="138"/>
+      <c r="B80" s="140"/>
+      <c r="C80" s="141"/>
       <c r="D80" s="139"/>
-      <c r="E80" s="140"/>
+      <c r="E80" s="138"/>
       <c r="F80" s="8">
         <v>246</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="142"/>
-      <c r="B81" s="143"/>
-      <c r="C81" s="138"/>
+      <c r="B81" s="140"/>
+      <c r="C81" s="141"/>
       <c r="D81" s="139">
         <v>249</v>
       </c>
-      <c r="E81" s="140">
+      <c r="E81" s="138">
         <v>249</v>
       </c>
       <c r="F81" s="8">
@@ -7620,20 +7620,20 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="142"/>
-      <c r="B82" s="143"/>
-      <c r="C82" s="138"/>
+      <c r="B82" s="140"/>
+      <c r="C82" s="141"/>
       <c r="D82" s="139"/>
-      <c r="E82" s="140"/>
+      <c r="E82" s="138"/>
       <c r="F82" s="8">
         <v>252</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="142"/>
-      <c r="B83" s="143"/>
-      <c r="C83" s="138"/>
+      <c r="B83" s="140"/>
+      <c r="C83" s="141"/>
       <c r="D83" s="139"/>
-      <c r="E83" s="140">
+      <c r="E83" s="138">
         <v>255</v>
       </c>
       <c r="F83" s="8">
@@ -7642,26 +7642,26 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="142"/>
-      <c r="B84" s="143"/>
-      <c r="C84" s="138"/>
+      <c r="B84" s="140"/>
+      <c r="C84" s="141"/>
       <c r="D84" s="139"/>
-      <c r="E84" s="140"/>
+      <c r="E84" s="138"/>
       <c r="F84" s="8">
         <v>258</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="142"/>
-      <c r="B85" s="143">
+      <c r="B85" s="140">
         <v>270</v>
       </c>
-      <c r="C85" s="138">
+      <c r="C85" s="141">
         <v>270</v>
       </c>
       <c r="D85" s="139">
         <v>261</v>
       </c>
-      <c r="E85" s="140">
+      <c r="E85" s="138">
         <v>261</v>
       </c>
       <c r="F85" s="8">
@@ -7670,20 +7670,20 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="142"/>
-      <c r="B86" s="143"/>
-      <c r="C86" s="138"/>
+      <c r="B86" s="140"/>
+      <c r="C86" s="141"/>
       <c r="D86" s="139"/>
-      <c r="E86" s="140"/>
+      <c r="E86" s="138"/>
       <c r="F86" s="8">
         <v>264</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="142"/>
-      <c r="B87" s="143"/>
-      <c r="C87" s="138"/>
+      <c r="B87" s="140"/>
+      <c r="C87" s="141"/>
       <c r="D87" s="139"/>
-      <c r="E87" s="140">
+      <c r="E87" s="138">
         <v>267</v>
       </c>
       <c r="F87" s="8">
@@ -7692,22 +7692,22 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="142"/>
-      <c r="B88" s="143"/>
-      <c r="C88" s="138"/>
+      <c r="B88" s="140"/>
+      <c r="C88" s="141"/>
       <c r="D88" s="139"/>
-      <c r="E88" s="140"/>
+      <c r="E88" s="138"/>
       <c r="F88" s="8">
         <v>271</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="142"/>
-      <c r="B89" s="143"/>
-      <c r="C89" s="138"/>
+      <c r="B89" s="140"/>
+      <c r="C89" s="141"/>
       <c r="D89" s="139">
         <v>274</v>
       </c>
-      <c r="E89" s="140">
+      <c r="E89" s="138">
         <v>274</v>
       </c>
       <c r="F89" s="8">
@@ -7716,20 +7716,20 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="142"/>
-      <c r="B90" s="143"/>
-      <c r="C90" s="138"/>
+      <c r="B90" s="140"/>
+      <c r="C90" s="141"/>
       <c r="D90" s="139"/>
-      <c r="E90" s="140"/>
+      <c r="E90" s="138"/>
       <c r="F90" s="8">
         <v>277</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="142"/>
-      <c r="B91" s="143"/>
-      <c r="C91" s="138"/>
+      <c r="B91" s="140"/>
+      <c r="C91" s="141"/>
       <c r="D91" s="139"/>
-      <c r="E91" s="140">
+      <c r="E91" s="138">
         <v>280</v>
       </c>
       <c r="F91" s="8">
@@ -7738,24 +7738,24 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="142"/>
-      <c r="B92" s="143"/>
-      <c r="C92" s="138"/>
+      <c r="B92" s="140"/>
+      <c r="C92" s="141"/>
       <c r="D92" s="139"/>
-      <c r="E92" s="140"/>
+      <c r="E92" s="138"/>
       <c r="F92" s="8">
         <v>284</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="142"/>
-      <c r="B93" s="143"/>
-      <c r="C93" s="138">
+      <c r="B93" s="140"/>
+      <c r="C93" s="141">
         <v>300</v>
       </c>
       <c r="D93" s="139">
         <v>287</v>
       </c>
-      <c r="E93" s="140">
+      <c r="E93" s="138">
         <v>287</v>
       </c>
       <c r="F93" s="8">
@@ -7764,20 +7764,20 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="142"/>
-      <c r="B94" s="143"/>
-      <c r="C94" s="138"/>
+      <c r="B94" s="140"/>
+      <c r="C94" s="141"/>
       <c r="D94" s="139"/>
-      <c r="E94" s="140"/>
+      <c r="E94" s="138"/>
       <c r="F94" s="8">
         <v>291</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="142"/>
-      <c r="B95" s="143"/>
-      <c r="C95" s="138"/>
+      <c r="B95" s="140"/>
+      <c r="C95" s="141"/>
       <c r="D95" s="139"/>
-      <c r="E95" s="140">
+      <c r="E95" s="138">
         <v>294</v>
       </c>
       <c r="F95" s="8">
@@ -7786,22 +7786,22 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="142"/>
-      <c r="B96" s="143"/>
-      <c r="C96" s="138"/>
+      <c r="B96" s="140"/>
+      <c r="C96" s="141"/>
       <c r="D96" s="139"/>
-      <c r="E96" s="140"/>
+      <c r="E96" s="138"/>
       <c r="F96" s="8">
         <v>298</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="142"/>
-      <c r="B97" s="143"/>
-      <c r="C97" s="138"/>
+      <c r="B97" s="140"/>
+      <c r="C97" s="141"/>
       <c r="D97" s="139">
         <v>301</v>
       </c>
-      <c r="E97" s="140">
+      <c r="E97" s="138">
         <v>301</v>
       </c>
       <c r="F97" s="8">
@@ -7810,20 +7810,20 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="142"/>
-      <c r="B98" s="143"/>
-      <c r="C98" s="138"/>
+      <c r="B98" s="140"/>
+      <c r="C98" s="141"/>
       <c r="D98" s="139"/>
-      <c r="E98" s="140"/>
+      <c r="E98" s="138"/>
       <c r="F98" s="8">
         <v>305</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="142"/>
-      <c r="B99" s="143"/>
-      <c r="C99" s="138"/>
+      <c r="B99" s="140"/>
+      <c r="C99" s="141"/>
       <c r="D99" s="139"/>
-      <c r="E99" s="140">
+      <c r="E99" s="138">
         <v>309</v>
       </c>
       <c r="F99" s="8">
@@ -7832,10 +7832,10 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="142"/>
-      <c r="B100" s="143"/>
-      <c r="C100" s="138"/>
+      <c r="B100" s="140"/>
+      <c r="C100" s="141"/>
       <c r="D100" s="139"/>
-      <c r="E100" s="140"/>
+      <c r="E100" s="138"/>
       <c r="F100" s="8">
         <v>312</v>
       </c>
@@ -7844,16 +7844,16 @@
       <c r="A101" s="142">
         <v>330</v>
       </c>
-      <c r="B101" s="143">
+      <c r="B101" s="140">
         <v>330</v>
       </c>
-      <c r="C101" s="138">
+      <c r="C101" s="141">
         <v>330</v>
       </c>
       <c r="D101" s="139">
         <v>316</v>
       </c>
-      <c r="E101" s="140">
+      <c r="E101" s="138">
         <v>316</v>
       </c>
       <c r="F101" s="8">
@@ -7862,20 +7862,20 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="142"/>
-      <c r="B102" s="143"/>
-      <c r="C102" s="138"/>
+      <c r="B102" s="140"/>
+      <c r="C102" s="141"/>
       <c r="D102" s="139"/>
-      <c r="E102" s="140"/>
+      <c r="E102" s="138"/>
       <c r="F102" s="8">
         <v>320</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="142"/>
-      <c r="B103" s="143"/>
-      <c r="C103" s="138"/>
+      <c r="B103" s="140"/>
+      <c r="C103" s="141"/>
       <c r="D103" s="139"/>
-      <c r="E103" s="140">
+      <c r="E103" s="138">
         <v>324</v>
       </c>
       <c r="F103" s="8">
@@ -7884,22 +7884,22 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="142"/>
-      <c r="B104" s="143"/>
-      <c r="C104" s="138"/>
+      <c r="B104" s="140"/>
+      <c r="C104" s="141"/>
       <c r="D104" s="139"/>
-      <c r="E104" s="140"/>
+      <c r="E104" s="138"/>
       <c r="F104" s="8">
         <v>328</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="142"/>
-      <c r="B105" s="143"/>
-      <c r="C105" s="138"/>
+      <c r="B105" s="140"/>
+      <c r="C105" s="141"/>
       <c r="D105" s="139">
         <v>332</v>
       </c>
-      <c r="E105" s="140">
+      <c r="E105" s="138">
         <v>332</v>
       </c>
       <c r="F105" s="8">
@@ -7908,20 +7908,20 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="142"/>
-      <c r="B106" s="143"/>
-      <c r="C106" s="138"/>
+      <c r="B106" s="140"/>
+      <c r="C106" s="141"/>
       <c r="D106" s="139"/>
-      <c r="E106" s="140"/>
+      <c r="E106" s="138"/>
       <c r="F106" s="8">
         <v>336</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="142"/>
-      <c r="B107" s="143"/>
-      <c r="C107" s="138"/>
+      <c r="B107" s="140"/>
+      <c r="C107" s="141"/>
       <c r="D107" s="139"/>
-      <c r="E107" s="140">
+      <c r="E107" s="138">
         <v>340</v>
       </c>
       <c r="F107" s="8">
@@ -7930,24 +7930,24 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="142"/>
-      <c r="B108" s="143"/>
-      <c r="C108" s="138"/>
+      <c r="B108" s="140"/>
+      <c r="C108" s="141"/>
       <c r="D108" s="139"/>
-      <c r="E108" s="140"/>
+      <c r="E108" s="138"/>
       <c r="F108" s="8">
         <v>344</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="142"/>
-      <c r="B109" s="143"/>
-      <c r="C109" s="138">
+      <c r="B109" s="140"/>
+      <c r="C109" s="141">
         <v>360</v>
       </c>
       <c r="D109" s="139">
         <v>348</v>
       </c>
-      <c r="E109" s="140">
+      <c r="E109" s="138">
         <v>348</v>
       </c>
       <c r="F109" s="8">
@@ -7956,20 +7956,20 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="142"/>
-      <c r="B110" s="143"/>
-      <c r="C110" s="138"/>
+      <c r="B110" s="140"/>
+      <c r="C110" s="141"/>
       <c r="D110" s="139"/>
-      <c r="E110" s="140"/>
+      <c r="E110" s="138"/>
       <c r="F110" s="8">
         <v>352</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="142"/>
-      <c r="B111" s="143"/>
-      <c r="C111" s="138"/>
+      <c r="B111" s="140"/>
+      <c r="C111" s="141"/>
       <c r="D111" s="139"/>
-      <c r="E111" s="140">
+      <c r="E111" s="138">
         <v>357</v>
       </c>
       <c r="F111" s="8">
@@ -7978,22 +7978,22 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="142"/>
-      <c r="B112" s="143"/>
-      <c r="C112" s="138"/>
+      <c r="B112" s="140"/>
+      <c r="C112" s="141"/>
       <c r="D112" s="139"/>
-      <c r="E112" s="140"/>
+      <c r="E112" s="138"/>
       <c r="F112" s="8">
         <v>361</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="142"/>
-      <c r="B113" s="143"/>
-      <c r="C113" s="138"/>
+      <c r="B113" s="140"/>
+      <c r="C113" s="141"/>
       <c r="D113" s="139">
         <v>365</v>
       </c>
-      <c r="E113" s="140">
+      <c r="E113" s="138">
         <v>365</v>
       </c>
       <c r="F113" s="8">
@@ -8002,20 +8002,20 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="142"/>
-      <c r="B114" s="143"/>
-      <c r="C114" s="138"/>
+      <c r="B114" s="140"/>
+      <c r="C114" s="141"/>
       <c r="D114" s="139"/>
-      <c r="E114" s="140"/>
+      <c r="E114" s="138"/>
       <c r="F114" s="8">
         <v>370</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="142"/>
-      <c r="B115" s="143"/>
-      <c r="C115" s="138"/>
+      <c r="B115" s="140"/>
+      <c r="C115" s="141"/>
       <c r="D115" s="139"/>
-      <c r="E115" s="140">
+      <c r="E115" s="138">
         <v>374</v>
       </c>
       <c r="F115" s="8">
@@ -8024,26 +8024,26 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="142"/>
-      <c r="B116" s="143"/>
-      <c r="C116" s="138"/>
+      <c r="B116" s="140"/>
+      <c r="C116" s="141"/>
       <c r="D116" s="139"/>
-      <c r="E116" s="140"/>
+      <c r="E116" s="138"/>
       <c r="F116" s="8">
         <v>379</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="142"/>
-      <c r="B117" s="143">
+      <c r="B117" s="140">
         <v>390</v>
       </c>
-      <c r="C117" s="138">
+      <c r="C117" s="141">
         <v>390</v>
       </c>
       <c r="D117" s="139">
         <v>383</v>
       </c>
-      <c r="E117" s="140">
+      <c r="E117" s="138">
         <v>383</v>
       </c>
       <c r="F117" s="8">
@@ -8052,20 +8052,20 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="142"/>
-      <c r="B118" s="143"/>
-      <c r="C118" s="138"/>
+      <c r="B118" s="140"/>
+      <c r="C118" s="141"/>
       <c r="D118" s="139"/>
-      <c r="E118" s="140"/>
+      <c r="E118" s="138"/>
       <c r="F118" s="8">
         <v>388</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="142"/>
-      <c r="B119" s="143"/>
-      <c r="C119" s="138"/>
+      <c r="B119" s="140"/>
+      <c r="C119" s="141"/>
       <c r="D119" s="139"/>
-      <c r="E119" s="140">
+      <c r="E119" s="138">
         <v>392</v>
       </c>
       <c r="F119" s="8">
@@ -8074,22 +8074,22 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="142"/>
-      <c r="B120" s="143"/>
-      <c r="C120" s="138"/>
+      <c r="B120" s="140"/>
+      <c r="C120" s="141"/>
       <c r="D120" s="139"/>
-      <c r="E120" s="140"/>
+      <c r="E120" s="138"/>
       <c r="F120" s="8">
         <v>397</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="142"/>
-      <c r="B121" s="143"/>
-      <c r="C121" s="138"/>
+      <c r="B121" s="140"/>
+      <c r="C121" s="141"/>
       <c r="D121" s="139">
         <v>402</v>
       </c>
-      <c r="E121" s="140">
+      <c r="E121" s="138">
         <v>402</v>
       </c>
       <c r="F121" s="8">
@@ -8098,20 +8098,20 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="142"/>
-      <c r="B122" s="143"/>
-      <c r="C122" s="138"/>
+      <c r="B122" s="140"/>
+      <c r="C122" s="141"/>
       <c r="D122" s="139"/>
-      <c r="E122" s="140"/>
+      <c r="E122" s="138"/>
       <c r="F122" s="8">
         <v>407</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="142"/>
-      <c r="B123" s="143"/>
-      <c r="C123" s="138"/>
+      <c r="B123" s="140"/>
+      <c r="C123" s="141"/>
       <c r="D123" s="139"/>
-      <c r="E123" s="140">
+      <c r="E123" s="138">
         <v>412</v>
       </c>
       <c r="F123" s="8">
@@ -8120,24 +8120,24 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="142"/>
-      <c r="B124" s="143"/>
-      <c r="C124" s="138"/>
+      <c r="B124" s="140"/>
+      <c r="C124" s="141"/>
       <c r="D124" s="139"/>
-      <c r="E124" s="140"/>
+      <c r="E124" s="138"/>
       <c r="F124" s="8">
         <v>417</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="142"/>
-      <c r="B125" s="143"/>
-      <c r="C125" s="138">
+      <c r="B125" s="140"/>
+      <c r="C125" s="141">
         <v>430</v>
       </c>
       <c r="D125" s="139">
         <v>422</v>
       </c>
-      <c r="E125" s="140">
+      <c r="E125" s="138">
         <v>422</v>
       </c>
       <c r="F125" s="8">
@@ -8146,20 +8146,20 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="142"/>
-      <c r="B126" s="143"/>
-      <c r="C126" s="138"/>
+      <c r="B126" s="140"/>
+      <c r="C126" s="141"/>
       <c r="D126" s="139"/>
-      <c r="E126" s="140"/>
+      <c r="E126" s="138"/>
       <c r="F126" s="8">
         <v>427</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="142"/>
-      <c r="B127" s="143"/>
-      <c r="C127" s="138"/>
+      <c r="B127" s="140"/>
+      <c r="C127" s="141"/>
       <c r="D127" s="139"/>
-      <c r="E127" s="140">
+      <c r="E127" s="138">
         <v>432</v>
       </c>
       <c r="F127" s="8">
@@ -8168,22 +8168,22 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="142"/>
-      <c r="B128" s="143"/>
-      <c r="C128" s="138"/>
+      <c r="B128" s="140"/>
+      <c r="C128" s="141"/>
       <c r="D128" s="139"/>
-      <c r="E128" s="140"/>
+      <c r="E128" s="138"/>
       <c r="F128" s="8">
         <v>437</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="142"/>
-      <c r="B129" s="143"/>
-      <c r="C129" s="138"/>
+      <c r="B129" s="140"/>
+      <c r="C129" s="141"/>
       <c r="D129" s="139">
         <v>442</v>
       </c>
-      <c r="E129" s="140">
+      <c r="E129" s="138">
         <v>442</v>
       </c>
       <c r="F129" s="8">
@@ -8192,20 +8192,20 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="142"/>
-      <c r="B130" s="143"/>
-      <c r="C130" s="138"/>
+      <c r="B130" s="140"/>
+      <c r="C130" s="141"/>
       <c r="D130" s="139"/>
-      <c r="E130" s="140"/>
+      <c r="E130" s="138"/>
       <c r="F130" s="8">
         <v>448</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="142"/>
-      <c r="B131" s="143"/>
-      <c r="C131" s="138"/>
+      <c r="B131" s="140"/>
+      <c r="C131" s="141"/>
       <c r="D131" s="139"/>
-      <c r="E131" s="140">
+      <c r="E131" s="138">
         <v>453</v>
       </c>
       <c r="F131" s="8">
@@ -8214,10 +8214,10 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="142"/>
-      <c r="B132" s="143"/>
-      <c r="C132" s="138"/>
+      <c r="B132" s="140"/>
+      <c r="C132" s="141"/>
       <c r="D132" s="139"/>
-      <c r="E132" s="140"/>
+      <c r="E132" s="138"/>
       <c r="F132" s="8">
         <v>459</v>
       </c>
@@ -8226,16 +8226,16 @@
       <c r="A133" s="142">
         <v>470</v>
       </c>
-      <c r="B133" s="143">
+      <c r="B133" s="140">
         <v>470</v>
       </c>
-      <c r="C133" s="138">
+      <c r="C133" s="141">
         <v>470</v>
       </c>
       <c r="D133" s="139">
         <v>464</v>
       </c>
-      <c r="E133" s="140">
+      <c r="E133" s="138">
         <v>464</v>
       </c>
       <c r="F133" s="8">
@@ -8244,20 +8244,20 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="142"/>
-      <c r="B134" s="143"/>
-      <c r="C134" s="138"/>
+      <c r="B134" s="140"/>
+      <c r="C134" s="141"/>
       <c r="D134" s="139"/>
-      <c r="E134" s="140"/>
+      <c r="E134" s="138"/>
       <c r="F134" s="8">
         <v>470</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="142"/>
-      <c r="B135" s="143"/>
-      <c r="C135" s="138"/>
+      <c r="B135" s="140"/>
+      <c r="C135" s="141"/>
       <c r="D135" s="139"/>
-      <c r="E135" s="140">
+      <c r="E135" s="138">
         <v>475</v>
       </c>
       <c r="F135" s="8">
@@ -8266,22 +8266,22 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="142"/>
-      <c r="B136" s="143"/>
-      <c r="C136" s="138"/>
+      <c r="B136" s="140"/>
+      <c r="C136" s="141"/>
       <c r="D136" s="139"/>
-      <c r="E136" s="140"/>
+      <c r="E136" s="138"/>
       <c r="F136" s="8">
         <v>481</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="142"/>
-      <c r="B137" s="143"/>
-      <c r="C137" s="138"/>
+      <c r="B137" s="140"/>
+      <c r="C137" s="141"/>
       <c r="D137" s="139">
         <v>487</v>
       </c>
-      <c r="E137" s="140">
+      <c r="E137" s="138">
         <v>487</v>
       </c>
       <c r="F137" s="8">
@@ -8290,20 +8290,20 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="142"/>
-      <c r="B138" s="143"/>
-      <c r="C138" s="138"/>
+      <c r="B138" s="140"/>
+      <c r="C138" s="141"/>
       <c r="D138" s="139"/>
-      <c r="E138" s="140"/>
+      <c r="E138" s="138"/>
       <c r="F138" s="8">
         <v>493</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="142"/>
-      <c r="B139" s="143"/>
-      <c r="C139" s="138"/>
+      <c r="B139" s="140"/>
+      <c r="C139" s="141"/>
       <c r="D139" s="139"/>
-      <c r="E139" s="140">
+      <c r="E139" s="138">
         <v>499</v>
       </c>
       <c r="F139" s="8">
@@ -8312,24 +8312,24 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="142"/>
-      <c r="B140" s="143"/>
-      <c r="C140" s="138"/>
+      <c r="B140" s="140"/>
+      <c r="C140" s="141"/>
       <c r="D140" s="139"/>
-      <c r="E140" s="140"/>
+      <c r="E140" s="138"/>
       <c r="F140" s="8">
         <v>505</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="142"/>
-      <c r="B141" s="143"/>
-      <c r="C141" s="138">
+      <c r="B141" s="140"/>
+      <c r="C141" s="141">
         <v>510</v>
       </c>
       <c r="D141" s="139">
         <v>511</v>
       </c>
-      <c r="E141" s="140">
+      <c r="E141" s="138">
         <v>511</v>
       </c>
       <c r="F141" s="8">
@@ -8338,20 +8338,20 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="142"/>
-      <c r="B142" s="143"/>
-      <c r="C142" s="138"/>
+      <c r="B142" s="140"/>
+      <c r="C142" s="141"/>
       <c r="D142" s="139"/>
-      <c r="E142" s="140"/>
+      <c r="E142" s="138"/>
       <c r="F142" s="8">
         <v>517</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="142"/>
-      <c r="B143" s="143"/>
-      <c r="C143" s="138"/>
+      <c r="B143" s="140"/>
+      <c r="C143" s="141"/>
       <c r="D143" s="139"/>
-      <c r="E143" s="140">
+      <c r="E143" s="138">
         <v>523</v>
       </c>
       <c r="F143" s="8">
@@ -8360,22 +8360,22 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="142"/>
-      <c r="B144" s="143"/>
-      <c r="C144" s="138"/>
+      <c r="B144" s="140"/>
+      <c r="C144" s="141"/>
       <c r="D144" s="139"/>
-      <c r="E144" s="140"/>
+      <c r="E144" s="138"/>
       <c r="F144" s="8">
         <v>530</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="142"/>
-      <c r="B145" s="143"/>
-      <c r="C145" s="138"/>
+      <c r="B145" s="140"/>
+      <c r="C145" s="141"/>
       <c r="D145" s="139">
         <v>536</v>
       </c>
-      <c r="E145" s="140">
+      <c r="E145" s="138">
         <v>536</v>
       </c>
       <c r="F145" s="8">
@@ -8384,20 +8384,20 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="142"/>
-      <c r="B146" s="143"/>
-      <c r="C146" s="138"/>
+      <c r="B146" s="140"/>
+      <c r="C146" s="141"/>
       <c r="D146" s="139"/>
-      <c r="E146" s="140"/>
+      <c r="E146" s="138"/>
       <c r="F146" s="8">
         <v>542</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="142"/>
-      <c r="B147" s="143"/>
-      <c r="C147" s="138"/>
+      <c r="B147" s="140"/>
+      <c r="C147" s="141"/>
       <c r="D147" s="139"/>
-      <c r="E147" s="140">
+      <c r="E147" s="138">
         <v>549</v>
       </c>
       <c r="F147" s="8">
@@ -8406,26 +8406,26 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="142"/>
-      <c r="B148" s="143"/>
-      <c r="C148" s="138"/>
+      <c r="B148" s="140"/>
+      <c r="C148" s="141"/>
       <c r="D148" s="139"/>
-      <c r="E148" s="140"/>
+      <c r="E148" s="138"/>
       <c r="F148" s="8">
         <v>556</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="142"/>
-      <c r="B149" s="143">
+      <c r="B149" s="140">
         <v>560</v>
       </c>
-      <c r="C149" s="138">
+      <c r="C149" s="141">
         <v>560</v>
       </c>
       <c r="D149" s="139">
         <v>562</v>
       </c>
-      <c r="E149" s="140">
+      <c r="E149" s="138">
         <v>562</v>
       </c>
       <c r="F149" s="8">
@@ -8434,20 +8434,20 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="142"/>
-      <c r="B150" s="143"/>
-      <c r="C150" s="138"/>
+      <c r="B150" s="140"/>
+      <c r="C150" s="141"/>
       <c r="D150" s="139"/>
-      <c r="E150" s="140"/>
+      <c r="E150" s="138"/>
       <c r="F150" s="8">
         <v>569</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="142"/>
-      <c r="B151" s="143"/>
-      <c r="C151" s="138"/>
+      <c r="B151" s="140"/>
+      <c r="C151" s="141"/>
       <c r="D151" s="139"/>
-      <c r="E151" s="140">
+      <c r="E151" s="138">
         <v>576</v>
       </c>
       <c r="F151" s="8">
@@ -8456,22 +8456,22 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="142"/>
-      <c r="B152" s="143"/>
-      <c r="C152" s="138"/>
+      <c r="B152" s="140"/>
+      <c r="C152" s="141"/>
       <c r="D152" s="139"/>
-      <c r="E152" s="140"/>
+      <c r="E152" s="138"/>
       <c r="F152" s="8">
         <v>583</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="142"/>
-      <c r="B153" s="143"/>
-      <c r="C153" s="138"/>
+      <c r="B153" s="140"/>
+      <c r="C153" s="141"/>
       <c r="D153" s="139">
         <v>590</v>
       </c>
-      <c r="E153" s="140">
+      <c r="E153" s="138">
         <v>590</v>
       </c>
       <c r="F153" s="8">
@@ -8480,20 +8480,20 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="142"/>
-      <c r="B154" s="143"/>
-      <c r="C154" s="138"/>
+      <c r="B154" s="140"/>
+      <c r="C154" s="141"/>
       <c r="D154" s="139"/>
-      <c r="E154" s="140"/>
+      <c r="E154" s="138"/>
       <c r="F154" s="8">
         <v>597</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="142"/>
-      <c r="B155" s="143"/>
-      <c r="C155" s="138"/>
+      <c r="B155" s="140"/>
+      <c r="C155" s="141"/>
       <c r="D155" s="139"/>
-      <c r="E155" s="140">
+      <c r="E155" s="138">
         <v>604</v>
       </c>
       <c r="F155" s="8">
@@ -8502,24 +8502,24 @@
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="142"/>
-      <c r="B156" s="143"/>
-      <c r="C156" s="138"/>
+      <c r="B156" s="140"/>
+      <c r="C156" s="141"/>
       <c r="D156" s="139"/>
-      <c r="E156" s="140"/>
+      <c r="E156" s="138"/>
       <c r="F156" s="8">
         <v>612</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="142"/>
-      <c r="B157" s="143"/>
-      <c r="C157" s="138">
+      <c r="B157" s="140"/>
+      <c r="C157" s="141">
         <v>620</v>
       </c>
       <c r="D157" s="139">
         <v>619</v>
       </c>
-      <c r="E157" s="140">
+      <c r="E157" s="138">
         <v>619</v>
       </c>
       <c r="F157" s="8">
@@ -8528,20 +8528,20 @@
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="142"/>
-      <c r="B158" s="143"/>
-      <c r="C158" s="138"/>
+      <c r="B158" s="140"/>
+      <c r="C158" s="141"/>
       <c r="D158" s="139"/>
-      <c r="E158" s="140"/>
+      <c r="E158" s="138"/>
       <c r="F158" s="8">
         <v>626</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="142"/>
-      <c r="B159" s="143"/>
-      <c r="C159" s="138"/>
+      <c r="B159" s="140"/>
+      <c r="C159" s="141"/>
       <c r="D159" s="139"/>
-      <c r="E159" s="140">
+      <c r="E159" s="138">
         <v>634</v>
       </c>
       <c r="F159" s="8">
@@ -8550,22 +8550,22 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="142"/>
-      <c r="B160" s="143"/>
-      <c r="C160" s="138"/>
+      <c r="B160" s="140"/>
+      <c r="C160" s="141"/>
       <c r="D160" s="139"/>
-      <c r="E160" s="140"/>
+      <c r="E160" s="138"/>
       <c r="F160" s="8">
         <v>642</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="142"/>
-      <c r="B161" s="143"/>
-      <c r="C161" s="138"/>
+      <c r="B161" s="140"/>
+      <c r="C161" s="141"/>
       <c r="D161" s="139">
         <v>649</v>
       </c>
-      <c r="E161" s="140">
+      <c r="E161" s="138">
         <v>649</v>
       </c>
       <c r="F161" s="8">
@@ -8574,20 +8574,20 @@
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="142"/>
-      <c r="B162" s="143"/>
-      <c r="C162" s="138"/>
+      <c r="B162" s="140"/>
+      <c r="C162" s="141"/>
       <c r="D162" s="139"/>
-      <c r="E162" s="140"/>
+      <c r="E162" s="138"/>
       <c r="F162" s="8">
         <v>657</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="142"/>
-      <c r="B163" s="143"/>
-      <c r="C163" s="138"/>
+      <c r="B163" s="140"/>
+      <c r="C163" s="141"/>
       <c r="D163" s="139"/>
-      <c r="E163" s="140">
+      <c r="E163" s="138">
         <v>665</v>
       </c>
       <c r="F163" s="8">
@@ -8596,10 +8596,10 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="142"/>
-      <c r="B164" s="143"/>
-      <c r="C164" s="138"/>
+      <c r="B164" s="140"/>
+      <c r="C164" s="141"/>
       <c r="D164" s="139"/>
-      <c r="E164" s="140"/>
+      <c r="E164" s="138"/>
       <c r="F164" s="8">
         <v>673</v>
       </c>
@@ -8608,16 +8608,16 @@
       <c r="A165" s="142">
         <v>680</v>
       </c>
-      <c r="B165" s="143">
+      <c r="B165" s="140">
         <v>680</v>
       </c>
-      <c r="C165" s="138">
+      <c r="C165" s="141">
         <v>680</v>
       </c>
       <c r="D165" s="139">
         <v>681</v>
       </c>
-      <c r="E165" s="140">
+      <c r="E165" s="138">
         <v>681</v>
       </c>
       <c r="F165" s="8">
@@ -8626,20 +8626,20 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="142"/>
-      <c r="B166" s="143"/>
-      <c r="C166" s="138"/>
+      <c r="B166" s="140"/>
+      <c r="C166" s="141"/>
       <c r="D166" s="139"/>
-      <c r="E166" s="140"/>
+      <c r="E166" s="138"/>
       <c r="F166" s="8">
         <v>690</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="142"/>
-      <c r="B167" s="143"/>
-      <c r="C167" s="138"/>
+      <c r="B167" s="140"/>
+      <c r="C167" s="141"/>
       <c r="D167" s="139"/>
-      <c r="E167" s="140">
+      <c r="E167" s="138">
         <v>698</v>
       </c>
       <c r="F167" s="8">
@@ -8648,22 +8648,22 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="142"/>
-      <c r="B168" s="143"/>
-      <c r="C168" s="138"/>
+      <c r="B168" s="140"/>
+      <c r="C168" s="141"/>
       <c r="D168" s="139"/>
-      <c r="E168" s="140"/>
+      <c r="E168" s="138"/>
       <c r="F168" s="8">
         <v>706</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="142"/>
-      <c r="B169" s="143"/>
-      <c r="C169" s="138"/>
+      <c r="B169" s="140"/>
+      <c r="C169" s="141"/>
       <c r="D169" s="139">
         <v>715</v>
       </c>
-      <c r="E169" s="140">
+      <c r="E169" s="138">
         <v>715</v>
       </c>
       <c r="F169" s="8">
@@ -8672,20 +8672,20 @@
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="142"/>
-      <c r="B170" s="143"/>
-      <c r="C170" s="138"/>
+      <c r="B170" s="140"/>
+      <c r="C170" s="141"/>
       <c r="D170" s="139"/>
-      <c r="E170" s="140"/>
+      <c r="E170" s="138"/>
       <c r="F170" s="8">
         <v>723</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="142"/>
-      <c r="B171" s="143"/>
-      <c r="C171" s="138"/>
+      <c r="B171" s="140"/>
+      <c r="C171" s="141"/>
       <c r="D171" s="139"/>
-      <c r="E171" s="140">
+      <c r="E171" s="138">
         <v>732</v>
       </c>
       <c r="F171" s="8">
@@ -8694,24 +8694,24 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="142"/>
-      <c r="B172" s="143"/>
-      <c r="C172" s="138"/>
+      <c r="B172" s="140"/>
+      <c r="C172" s="141"/>
       <c r="D172" s="139"/>
-      <c r="E172" s="140"/>
+      <c r="E172" s="138"/>
       <c r="F172" s="8">
         <v>741</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="142"/>
-      <c r="B173" s="143"/>
-      <c r="C173" s="138">
+      <c r="B173" s="140"/>
+      <c r="C173" s="141">
         <v>750</v>
       </c>
       <c r="D173" s="139">
         <v>750</v>
       </c>
-      <c r="E173" s="140">
+      <c r="E173" s="138">
         <v>750</v>
       </c>
       <c r="F173" s="8">
@@ -8720,20 +8720,20 @@
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" s="142"/>
-      <c r="B174" s="143"/>
-      <c r="C174" s="138"/>
+      <c r="B174" s="140"/>
+      <c r="C174" s="141"/>
       <c r="D174" s="139"/>
-      <c r="E174" s="140"/>
+      <c r="E174" s="138"/>
       <c r="F174" s="8">
         <v>759</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="142"/>
-      <c r="B175" s="143"/>
-      <c r="C175" s="138"/>
+      <c r="B175" s="140"/>
+      <c r="C175" s="141"/>
       <c r="D175" s="139"/>
-      <c r="E175" s="140">
+      <c r="E175" s="138">
         <v>768</v>
       </c>
       <c r="F175" s="8">
@@ -8742,22 +8742,22 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="142"/>
-      <c r="B176" s="143"/>
-      <c r="C176" s="138"/>
+      <c r="B176" s="140"/>
+      <c r="C176" s="141"/>
       <c r="D176" s="139"/>
-      <c r="E176" s="140"/>
+      <c r="E176" s="138"/>
       <c r="F176" s="8">
         <v>777</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="142"/>
-      <c r="B177" s="143"/>
-      <c r="C177" s="138"/>
+      <c r="B177" s="140"/>
+      <c r="C177" s="141"/>
       <c r="D177" s="139">
         <v>787</v>
       </c>
-      <c r="E177" s="140">
+      <c r="E177" s="138">
         <v>787</v>
       </c>
       <c r="F177" s="8">
@@ -8766,20 +8766,20 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="142"/>
-      <c r="B178" s="143"/>
-      <c r="C178" s="138"/>
+      <c r="B178" s="140"/>
+      <c r="C178" s="141"/>
       <c r="D178" s="139"/>
-      <c r="E178" s="140"/>
+      <c r="E178" s="138"/>
       <c r="F178" s="8">
         <v>796</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="142"/>
-      <c r="B179" s="143"/>
-      <c r="C179" s="138"/>
+      <c r="B179" s="140"/>
+      <c r="C179" s="141"/>
       <c r="D179" s="139"/>
-      <c r="E179" s="140">
+      <c r="E179" s="138">
         <v>806</v>
       </c>
       <c r="F179" s="8">
@@ -8788,26 +8788,26 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="142"/>
-      <c r="B180" s="143"/>
-      <c r="C180" s="138"/>
+      <c r="B180" s="140"/>
+      <c r="C180" s="141"/>
       <c r="D180" s="139"/>
-      <c r="E180" s="140"/>
+      <c r="E180" s="138"/>
       <c r="F180" s="8">
         <v>816</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="142"/>
-      <c r="B181" s="143">
+      <c r="B181" s="140">
         <v>820</v>
       </c>
-      <c r="C181" s="138">
+      <c r="C181" s="141">
         <v>820</v>
       </c>
       <c r="D181" s="139">
         <v>825</v>
       </c>
-      <c r="E181" s="140">
+      <c r="E181" s="138">
         <v>825</v>
       </c>
       <c r="F181" s="8">
@@ -8816,20 +8816,20 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" s="142"/>
-      <c r="B182" s="143"/>
-      <c r="C182" s="138"/>
+      <c r="B182" s="140"/>
+      <c r="C182" s="141"/>
       <c r="D182" s="139"/>
-      <c r="E182" s="140"/>
+      <c r="E182" s="138"/>
       <c r="F182" s="8">
         <v>835</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="142"/>
-      <c r="B183" s="143"/>
-      <c r="C183" s="138"/>
+      <c r="B183" s="140"/>
+      <c r="C183" s="141"/>
       <c r="D183" s="139"/>
-      <c r="E183" s="140">
+      <c r="E183" s="138">
         <v>845</v>
       </c>
       <c r="F183" s="8">
@@ -8838,22 +8838,22 @@
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="142"/>
-      <c r="B184" s="143"/>
-      <c r="C184" s="138"/>
+      <c r="B184" s="140"/>
+      <c r="C184" s="141"/>
       <c r="D184" s="139"/>
-      <c r="E184" s="140"/>
+      <c r="E184" s="138"/>
       <c r="F184" s="8">
         <v>856</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" s="142"/>
-      <c r="B185" s="143"/>
-      <c r="C185" s="138"/>
+      <c r="B185" s="140"/>
+      <c r="C185" s="141"/>
       <c r="D185" s="139">
         <v>866</v>
       </c>
-      <c r="E185" s="140">
+      <c r="E185" s="138">
         <v>866</v>
       </c>
       <c r="F185" s="8">
@@ -8862,20 +8862,20 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" s="142"/>
-      <c r="B186" s="143"/>
-      <c r="C186" s="138"/>
+      <c r="B186" s="140"/>
+      <c r="C186" s="141"/>
       <c r="D186" s="139"/>
-      <c r="E186" s="140"/>
+      <c r="E186" s="138"/>
       <c r="F186" s="8">
         <v>876</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" s="142"/>
-      <c r="B187" s="143"/>
-      <c r="C187" s="138"/>
+      <c r="B187" s="140"/>
+      <c r="C187" s="141"/>
       <c r="D187" s="139"/>
-      <c r="E187" s="140">
+      <c r="E187" s="138">
         <v>887</v>
       </c>
       <c r="F187" s="8">
@@ -8884,24 +8884,24 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" s="142"/>
-      <c r="B188" s="143"/>
-      <c r="C188" s="138"/>
+      <c r="B188" s="140"/>
+      <c r="C188" s="141"/>
       <c r="D188" s="139"/>
-      <c r="E188" s="140"/>
+      <c r="E188" s="138"/>
       <c r="F188" s="8">
         <v>898</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" s="142"/>
-      <c r="B189" s="143"/>
-      <c r="C189" s="138">
+      <c r="B189" s="140"/>
+      <c r="C189" s="141">
         <v>910</v>
       </c>
       <c r="D189" s="139">
         <v>909</v>
       </c>
-      <c r="E189" s="140">
+      <c r="E189" s="138">
         <v>909</v>
       </c>
       <c r="F189" s="8">
@@ -8910,20 +8910,20 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" s="142"/>
-      <c r="B190" s="143"/>
-      <c r="C190" s="138"/>
+      <c r="B190" s="140"/>
+      <c r="C190" s="141"/>
       <c r="D190" s="139"/>
-      <c r="E190" s="140"/>
+      <c r="E190" s="138"/>
       <c r="F190" s="8">
         <v>920</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="142"/>
-      <c r="B191" s="143"/>
-      <c r="C191" s="138"/>
+      <c r="B191" s="140"/>
+      <c r="C191" s="141"/>
       <c r="D191" s="139"/>
-      <c r="E191" s="140">
+      <c r="E191" s="138">
         <v>931</v>
       </c>
       <c r="F191" s="8">
@@ -8932,22 +8932,22 @@
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" s="142"/>
-      <c r="B192" s="143"/>
-      <c r="C192" s="138"/>
+      <c r="B192" s="140"/>
+      <c r="C192" s="141"/>
       <c r="D192" s="139"/>
-      <c r="E192" s="140"/>
+      <c r="E192" s="138"/>
       <c r="F192" s="8">
         <v>942</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="142"/>
-      <c r="B193" s="143"/>
-      <c r="C193" s="138"/>
+      <c r="B193" s="140"/>
+      <c r="C193" s="141"/>
       <c r="D193" s="139">
         <v>953</v>
       </c>
-      <c r="E193" s="140">
+      <c r="E193" s="138">
         <v>953</v>
       </c>
       <c r="F193" s="8">
@@ -8956,20 +8956,20 @@
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" s="142"/>
-      <c r="B194" s="143"/>
-      <c r="C194" s="138"/>
+      <c r="B194" s="140"/>
+      <c r="C194" s="141"/>
       <c r="D194" s="139"/>
-      <c r="E194" s="140"/>
+      <c r="E194" s="138"/>
       <c r="F194" s="8">
         <v>965</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="142"/>
-      <c r="B195" s="143"/>
-      <c r="C195" s="138"/>
+      <c r="B195" s="140"/>
+      <c r="C195" s="141"/>
       <c r="D195" s="139"/>
-      <c r="E195" s="140">
+      <c r="E195" s="138">
         <v>976</v>
       </c>
       <c r="F195" s="8">
@@ -8978,33 +8978,162 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" s="142"/>
-      <c r="B196" s="143"/>
-      <c r="C196" s="138"/>
+      <c r="B196" s="140"/>
+      <c r="C196" s="141"/>
       <c r="D196" s="139"/>
-      <c r="E196" s="140"/>
+      <c r="E196" s="138"/>
       <c r="F196" s="8">
         <v>988</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="187">
-    <mergeCell ref="E177:E178"/>
-    <mergeCell ref="D189:D192"/>
-    <mergeCell ref="E189:E190"/>
-    <mergeCell ref="E191:E192"/>
-    <mergeCell ref="D193:D196"/>
-    <mergeCell ref="E193:E194"/>
-    <mergeCell ref="E195:E196"/>
-    <mergeCell ref="E179:E180"/>
-    <mergeCell ref="B181:B196"/>
-    <mergeCell ref="C181:C188"/>
-    <mergeCell ref="D181:D184"/>
-    <mergeCell ref="E181:E182"/>
-    <mergeCell ref="E183:E184"/>
-    <mergeCell ref="D185:D188"/>
-    <mergeCell ref="E185:E186"/>
-    <mergeCell ref="E187:E188"/>
-    <mergeCell ref="C189:C196"/>
+    <mergeCell ref="C13:C20"/>
+    <mergeCell ref="D13:D16"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="D17:D20"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:A36"/>
+    <mergeCell ref="B5:B20"/>
+    <mergeCell ref="C5:C12"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="A37:A68"/>
+    <mergeCell ref="B37:B52"/>
+    <mergeCell ref="C37:C44"/>
+    <mergeCell ref="D37:D40"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B21:B36"/>
+    <mergeCell ref="C21:C28"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C29:C36"/>
+    <mergeCell ref="D29:D32"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="D41:D44"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="D61:D64"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="D65:D68"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="B53:B68"/>
+    <mergeCell ref="C53:C60"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="D57:D60"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="C61:C68"/>
+    <mergeCell ref="D77:D80"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="D81:D84"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="A69:A100"/>
+    <mergeCell ref="B69:B84"/>
+    <mergeCell ref="C69:C76"/>
+    <mergeCell ref="D69:D72"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="D73:D76"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="C77:C84"/>
+    <mergeCell ref="E93:E94"/>
+    <mergeCell ref="E95:E96"/>
+    <mergeCell ref="D97:D100"/>
+    <mergeCell ref="E97:E98"/>
+    <mergeCell ref="E99:E100"/>
+    <mergeCell ref="A101:A132"/>
+    <mergeCell ref="B101:B116"/>
+    <mergeCell ref="C101:C108"/>
+    <mergeCell ref="D101:D104"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="B85:B100"/>
+    <mergeCell ref="C85:C92"/>
+    <mergeCell ref="D85:D88"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="E87:E88"/>
+    <mergeCell ref="D89:D92"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="E91:E92"/>
+    <mergeCell ref="C93:C100"/>
+    <mergeCell ref="D93:D96"/>
+    <mergeCell ref="E103:E104"/>
+    <mergeCell ref="D105:D108"/>
+    <mergeCell ref="E105:E106"/>
+    <mergeCell ref="E107:E108"/>
+    <mergeCell ref="C109:C116"/>
+    <mergeCell ref="D109:D112"/>
+    <mergeCell ref="E109:E110"/>
+    <mergeCell ref="E111:E112"/>
+    <mergeCell ref="D113:D116"/>
+    <mergeCell ref="E113:E114"/>
+    <mergeCell ref="D125:D128"/>
+    <mergeCell ref="E125:E126"/>
+    <mergeCell ref="E127:E128"/>
+    <mergeCell ref="D129:D132"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="E131:E132"/>
+    <mergeCell ref="E115:E116"/>
+    <mergeCell ref="B117:B132"/>
+    <mergeCell ref="C117:C124"/>
+    <mergeCell ref="D117:D120"/>
+    <mergeCell ref="E117:E118"/>
+    <mergeCell ref="E119:E120"/>
+    <mergeCell ref="D121:D124"/>
+    <mergeCell ref="E121:E122"/>
+    <mergeCell ref="E123:E124"/>
+    <mergeCell ref="C125:C132"/>
+    <mergeCell ref="D141:D144"/>
+    <mergeCell ref="E141:E142"/>
+    <mergeCell ref="E143:E144"/>
+    <mergeCell ref="D145:D148"/>
+    <mergeCell ref="E145:E146"/>
+    <mergeCell ref="E147:E148"/>
+    <mergeCell ref="A133:A164"/>
+    <mergeCell ref="B133:B148"/>
+    <mergeCell ref="C133:C140"/>
+    <mergeCell ref="D133:D136"/>
+    <mergeCell ref="E133:E134"/>
+    <mergeCell ref="E135:E136"/>
+    <mergeCell ref="D137:D140"/>
+    <mergeCell ref="E137:E138"/>
+    <mergeCell ref="E139:E140"/>
+    <mergeCell ref="C141:C148"/>
+    <mergeCell ref="E157:E158"/>
+    <mergeCell ref="E159:E160"/>
+    <mergeCell ref="D161:D164"/>
+    <mergeCell ref="E161:E162"/>
+    <mergeCell ref="E163:E164"/>
     <mergeCell ref="A165:A196"/>
     <mergeCell ref="B165:B180"/>
     <mergeCell ref="C165:C172"/>
@@ -9029,152 +9158,23 @@
     <mergeCell ref="E173:E174"/>
     <mergeCell ref="E175:E176"/>
     <mergeCell ref="D177:D180"/>
-    <mergeCell ref="D141:D144"/>
-    <mergeCell ref="E141:E142"/>
-    <mergeCell ref="E143:E144"/>
-    <mergeCell ref="D145:D148"/>
-    <mergeCell ref="E145:E146"/>
-    <mergeCell ref="E147:E148"/>
-    <mergeCell ref="A133:A164"/>
-    <mergeCell ref="B133:B148"/>
-    <mergeCell ref="C133:C140"/>
-    <mergeCell ref="D133:D136"/>
-    <mergeCell ref="E133:E134"/>
-    <mergeCell ref="E135:E136"/>
-    <mergeCell ref="D137:D140"/>
-    <mergeCell ref="E137:E138"/>
-    <mergeCell ref="E139:E140"/>
-    <mergeCell ref="C141:C148"/>
-    <mergeCell ref="E157:E158"/>
-    <mergeCell ref="E159:E160"/>
-    <mergeCell ref="D161:D164"/>
-    <mergeCell ref="E161:E162"/>
-    <mergeCell ref="E163:E164"/>
-    <mergeCell ref="E113:E114"/>
-    <mergeCell ref="D125:D128"/>
-    <mergeCell ref="E125:E126"/>
-    <mergeCell ref="E127:E128"/>
-    <mergeCell ref="D129:D132"/>
-    <mergeCell ref="E129:E130"/>
-    <mergeCell ref="E131:E132"/>
-    <mergeCell ref="E115:E116"/>
-    <mergeCell ref="B117:B132"/>
-    <mergeCell ref="C117:C124"/>
-    <mergeCell ref="D117:D120"/>
-    <mergeCell ref="E117:E118"/>
-    <mergeCell ref="E119:E120"/>
-    <mergeCell ref="D121:D124"/>
-    <mergeCell ref="E121:E122"/>
-    <mergeCell ref="E123:E124"/>
-    <mergeCell ref="C125:C132"/>
-    <mergeCell ref="A101:A132"/>
-    <mergeCell ref="B101:B116"/>
-    <mergeCell ref="C101:C108"/>
-    <mergeCell ref="D101:D104"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="B85:B100"/>
-    <mergeCell ref="C85:C92"/>
-    <mergeCell ref="D85:D88"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="E87:E88"/>
-    <mergeCell ref="D89:D92"/>
-    <mergeCell ref="E89:E90"/>
-    <mergeCell ref="E91:E92"/>
-    <mergeCell ref="C93:C100"/>
-    <mergeCell ref="D93:D96"/>
-    <mergeCell ref="E103:E104"/>
-    <mergeCell ref="D105:D108"/>
-    <mergeCell ref="E105:E106"/>
-    <mergeCell ref="E107:E108"/>
-    <mergeCell ref="C109:C116"/>
-    <mergeCell ref="D109:D112"/>
-    <mergeCell ref="E109:E110"/>
-    <mergeCell ref="E111:E112"/>
-    <mergeCell ref="D113:D116"/>
-    <mergeCell ref="D77:D80"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="D81:D84"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="A69:A100"/>
-    <mergeCell ref="B69:B84"/>
-    <mergeCell ref="C69:C76"/>
-    <mergeCell ref="D69:D72"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="D73:D76"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="C77:C84"/>
-    <mergeCell ref="E93:E94"/>
-    <mergeCell ref="E95:E96"/>
-    <mergeCell ref="D97:D100"/>
-    <mergeCell ref="E97:E98"/>
-    <mergeCell ref="E99:E100"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="D61:D64"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="D65:D68"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="B53:B68"/>
-    <mergeCell ref="C53:C60"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="D57:D60"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="C61:C68"/>
-    <mergeCell ref="A37:A68"/>
-    <mergeCell ref="B37:B52"/>
-    <mergeCell ref="C37:C44"/>
-    <mergeCell ref="D37:D40"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B21:B36"/>
-    <mergeCell ref="C21:C28"/>
-    <mergeCell ref="D21:D24"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="D25:D28"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C29:C36"/>
-    <mergeCell ref="D29:D32"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="D41:D44"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="D45:D48"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="D49:D52"/>
-    <mergeCell ref="C13:C20"/>
-    <mergeCell ref="D13:D16"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="D17:D20"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:A36"/>
-    <mergeCell ref="B5:B20"/>
-    <mergeCell ref="C5:C12"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="E177:E178"/>
+    <mergeCell ref="D189:D192"/>
+    <mergeCell ref="E189:E190"/>
+    <mergeCell ref="E191:E192"/>
+    <mergeCell ref="D193:D196"/>
+    <mergeCell ref="E193:E194"/>
+    <mergeCell ref="E195:E196"/>
+    <mergeCell ref="E179:E180"/>
+    <mergeCell ref="B181:B196"/>
+    <mergeCell ref="C181:C188"/>
+    <mergeCell ref="D181:D184"/>
+    <mergeCell ref="E181:E182"/>
+    <mergeCell ref="E183:E184"/>
+    <mergeCell ref="D185:D188"/>
+    <mergeCell ref="E185:E186"/>
+    <mergeCell ref="E187:E188"/>
+    <mergeCell ref="C189:C196"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>